<commit_message>
B&N rev6: W.R./FRT plan check - Cafe Work Room has no gypsum face (G/A-221), restroom W.R. confirmed, RFI-37; gates OK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev6.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev6.xlsx
@@ -1417,7 +1417,7 @@
     <t xml:space="preserve">FRP-1 (A-510 Room Finish Schedule: Cafe Work Room 104 FRP-1 all walls, Janitor 107 FRP, Cafe 103 below countertop): installer (A-002) and height not printed for the partitions. Not quantified - audit rev4 (AUDITORIA_rev4/COMPARATIVA_AUDITORIA.xlsx row 10), rev5: kept open.</t>
   </si>
   <si>
-    <t xml:space="preserve">FRP-1 SF = Cafe Work Room 104 faces 0 LF x FRP height + Janitor 107 faces 19.43 LF x FRP height (A-510); + PVC trim at FRP edges and inside corners</t>
+    <t xml:space="preserve">FRP-1 SF = Cafe Work Room 104 walls 87.52 LF (FRT plywood faces C-H1-N, C-H1-W, C-H2a, C-H2b x 2, C-E2; G/A-221, E/A-221) x FRP height + Janitor 107 faces 19.43 LF x FRP height (A-510); + PVC trim at FRP edges and inside corners</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-14</t>
@@ -1537,7 +1537,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): all 5/8" gyp bd on new walls AND GWB ceilings = Type X (A-001A Div 09 A.2; 4/A-121, 5/A-121 - rev2 (estimator decision 2026-10-25): ceilings to Type X); W.R. faces = 5/8" Type X W.R. No 5/8" regular remains.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied (rev5): 5/8" Type X 14,902.61 SF = walls 13,934.30 + GWB ceilings 859.08 (restroom ceilings moved to W.R., RFI-11) + vestibule box 105.5 + Grab &amp; Go soffit bottom 3.73; Type X W.R. 1,142.63 SF; 5/8" regular 0.</t>
+    <t xml:space="preserve">Applied (rev6): 5/8" Type X 14,902.61 SF = walls 13,934.30 + GWB ceilings 859.08 (restroom ceilings moved to W.R., RFI-11) + vestibule box 105.5 + Grab &amp; Go soffit bottom 3.73; Type X W.R. 1,142.63 SF; 5/8" regular 0.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-28</t>
@@ -1726,7 +1726,7 @@
     <t xml:space="preserve">Gypsum board on walls (layers per type)</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantified (rev5): 5/8" Type X 14,902.61 SF + 5/8" Type X W.R. 1,142.63 SF (A-410, A-001A, RFI-27, RFI-11); no 5/8" regular. Perimeter walls existing (RFI-01).</t>
+    <t xml:space="preserve">Quantified (rev6): 5/8" Type X 14,902.61 SF + 5/8" Type X W.R. 1,142.63 SF (A-410, A-001A, RFI-27, RFI-11); no 5/8" regular. Perimeter walls existing (RFI-01).</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-08</t>
@@ -1762,7 +1762,7 @@
     <t xml:space="preserve">Gypsum board ceilings</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantified (rev5): suspended GWB ceilings and soffits per A-121 (5/A-121, 4/A-121) and 2/A-221 = 981.38 SF: 5/8" Type X 859.08 SF + restroom ceilings 5/8" Type X W.R. 122.30 SF (A-410 Partition Notes 2).</t>
+    <t xml:space="preserve">Quantified (rev6): suspended GWB ceilings and soffits per A-121 (5/A-121, 4/A-121) and 2/A-221 = 981.38 SF: 5/8" Type X 859.08 SF + restroom ceilings 5/8" Type X W.R. 122.30 SF (A-410 Partition Notes 2).</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-12</t>

</xml_diff>

<commit_message>
B&N rev6 (WIP): RFI-37 resolved from A-225 / A-226A / A-510 - FRT plywood -951.75 SF; back-check pending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev6.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev6.xlsx
@@ -1159,7 +1159,7 @@
     <t xml:space="preserve">FRT plywood substrate (5/8 in.)</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: G/A-221, H/A-221, E/A-221, F/A-221, I/A-221, 1/A-226A, 6/A-226A, 3/A-221, A-410 (ALL PLYWOOD NEEDS TO BE FRT) | Breakdown [DERIVED]: C-H1-N-A-FRT 647.5 + C-H1-N-B-FRT 314.79 + C-H1-W-B-FRT 127.78 + C-H2a-A-FRT 127.78 + C-H2a-B-FRT 304.25 + C-H2b-A-FRT 20.47 + C-H2b-B-FRT 20.47 + C-H3a-A-FRT 102 + C-H3b-A-FRT 49.36 + C-E2-A-FRT 732.5 + C-F-A-FRT 81.5 + C-I-P.1-A-FRT 15 + C-I-A-FRT 34.65 + SS-N-WD1-FRT 91.08 + SS-E-WD1-FRT 40.48 + SS-GG-FRT 110.49 + C-I-E1-A-FRT 9.04 + C-I-E2-A-FRT 9.04 = 2,838.18 SF (strip length x height)</t>
+    <t xml:space="preserve">N/SHEET: G/A-221, H/A-221, E/A-221, F/A-221, I/A-221, 1/A-226A, 6/A-226A, 3/A-221, A-410 (ALL PLYWOOD NEEDS TO BE FRT) | Breakdown [DERIVED]: C-H1-N-B-FRT 314.79 + C-H1-W-B-FRT 127.78 + C-H2a-A-FRT 127.78 + C-H2b-A-FRT 20.47 + C-H2b-B-FRT 20.47 + C-H3a-A-FRT 102 + C-H3b-A-FRT 49.36 + C-E2-A-FRT 732.5 + C-F-A-FRT 81.5 + C-I-P.1-A-FRT 15 + C-I-A-FRT 34.65 + SS-N-WD1-FRT 91.08 + SS-E-WD1-FRT 40.48 + SS-GG-FRT 110.49 + C-I-E1-A-FRT 9.04 + C-I-E2-A-FRT 9.04 = 1,886.43 SF (strip length x height)</t>
   </si>
   <si>
     <t xml:space="preserve">FRT plywood substrate (3/4 in.)</t>
@@ -1624,10 +1624,10 @@
     <t xml:space="preserve">RFI-37</t>
   </si>
   <si>
-    <t xml:space="preserve">G/A-221 (types H1 / H2a) draws one board layer on the Sales Floor side (5/8" gypsum board) and one on the Cafe Work Room side (5/8" FRT plywood). The take-off carries 5/8" FRT plywood ALSO behind the gypsum board on the Sales / Cafe side of C-H1-N (25.90 x 25.0 = 647.50 SF) and C-H2a (12.17 x 25.0 = 304.25 SF) since rev0 (finish details "SEE SHEET A-225"). Confirm if plywood is required behind the GWB on those faces.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If not required: - 951.75 SF 5/8" FRT plywood (C-H1-N A 647.50 + C-H2a B 304.25); GWB unchanged.</t>
+    <t xml:space="preserve">CLOSED - resolved from the plan (rev6): the Sales / Cafe faces of C-H1-N and C-H2a are 5/8" gypsum board only. G/A-221 draws one layer on the Sales Floor side ("5/8" GYPSUM BOARD"); C-H1-N Sales face = Sales Area 101 PAINTED GYP. BD. (A-510); C-H2a Cafe face = PT-3 painted wall around door 3 (1/A-225 finish plan, 5/A-226A Cafe Service Line Elevation); the narrow WD-1 left of the door is the type I return C-I-P.1 (already carried). Evidence: investigacion_WR_FRT/ images 12-14.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied: - 951.75 SF 5/8" FRT plywood (C-H1-N A 25.90 x 25.0 = 647.50 + C-H2a B 12.17 x 25.0 = 304.25), carried since rev0; GWB on those faces unchanged.</t>
   </si>
   <si>
     <t xml:space="preserve">0 questions in total, asked ONE at a time in this order: floor plan (partition types A-Z), then the details the floor plan calls, in order</t>
@@ -1753,7 +1753,7 @@
     <t xml:space="preserve">FRT plywood sheathing / substrate</t>
   </si>
   <si>
-    <t xml:space="preserve">FRT plywood 5/8" 2,838.21 SF (Cafe types G, H, E2, F, I and Grab &amp; Go soffit 3/A-221; soffit faces 2/A-221) + 3/4" 370.46 SF (counters A/B, menu boards 4/A-226A, restroom backing 21/A-201, vestibule 4/A-210, 5/A-210, janitor 11/A-200) - breakdown in Material Summary</t>
+    <t xml:space="preserve">FRT plywood 5/8" 1,886.46 SF (Cafe types G, H, E2, F, I and Grab &amp; Go soffit 3/A-221; soffit faces 2/A-221) + 3/4" 370.46 SF (counters A/B, menu boards 4/A-226A, restroom backing 21/A-201, vestibule 4/A-210, 5/A-210, janitor 11/A-200) - breakdown in Material Summary</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-11</t>
@@ -1894,7 +1894,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "503c358310dabcee957eed4ec3cff89e4aa1601b1e5904822a6817eddb93d909", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "42f60b924cd916937587ab5c236dbca5be02769240c6b3d33aaa572a5bcf5ee1", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "604af291e542cf720eb181910415ee38c33ccfcb97e8ef821484cc1704df16ec", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "28f8aade70c6eb3d4395c4b0878064c24d9b64a63da5ca478fd6726965cdc239", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -6236,7 +6236,7 @@
         <v>357</v>
       </c>
       <c r="C29" s="0" t="n">
-        <v>2838.21</v>
+        <v>1886.46</v>
       </c>
       <c r="D29" s="0" t="n">
         <f aca="false">Inputs!$B$6</f>
@@ -6244,18 +6244,18 @@
       </c>
       <c r="E29" s="0" t="n">
         <f aca="false">C29*D29</f>
-        <v>170.2926</v>
+        <v>113.1876</v>
       </c>
       <c r="F29" s="0" t="n">
         <f aca="false">C29+E29</f>
-        <v>3008.5026</v>
+        <v>1999.6476</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>358</v>
       </c>
       <c r="H29" s="0" t="n">
         <f aca="false">ROUNDUP(F29/Inputs!$B$9,0)</f>
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="I29" s="0" t="s">
         <v>377</v>

</xml_diff>